<commit_message>
Import Lexique-only pilot and source cross-check evidence
</commit_message>
<xml_diff>
--- a/data/review-sheet.xlsx
+++ b/data/review-sheet.xlsx
@@ -634,7 +634,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>être (forme partagée), est (forme partagée), était, sont, es, été (forme partagée), suis (forme partagée), êtes (+33 more in data/pilot-300.json)</t>
+          <t>être (forme partagée), est (forme partagée), était, sont, es, été (forme partagée), suis (forme partagée), êtes (+33 autres formes)</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>avoir (forme partagée), a (forme partagée), ai, avait, as (forme partagée), ont, avez, eu (+38 more in data/pilot-300.json)</t>
+          <t>avoir (forme partagée), a (forme partagée), ai, avait, as (forme partagée), ont, avez, eu (+38 autres formes)</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>faire, fait (forme partagée), fais, faisait, faites (forme partagée), fit, font, fera (+32 more in data/pilot-300.json)</t>
+          <t>faire, fait (forme partagée), fais, faisait, faites (forme partagée), fit, font, fera (+32 autres formes)</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>aller (forme partagée), va (forme partagée), vais, allez (forme partagée), vas, allons, allait, vont (+31 more in data/pilot-300.json)</t>
+          <t>aller (forme partagée), va (forme partagée), vais, allez (forme partagée), vas, allons, allait, vont (+31 autres formes)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>dire (forme partagée), dit (forme partagée), dis, disait, dites (forme partagée), dirait, disais, disent (+24 more in data/pilot-300.json)</t>
+          <t>dire (forme partagée), dit (forme partagée), dis, disait, dites (forme partagée), dirait, disais, disent (+24 autres formes)</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>pouvoir (forme partagée), peux, peut, pu, pouvait, pourrait, pouvez, pourrais (+33 more in data/pilot-300.json)</t>
+          <t>pouvoir (forme partagée), peux, peut, pu, pouvait, pourrait, pouvez, pourrais (+33 autres formes)</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>vouloir (forme partagée), veux, veut, voulez (forme partagée), voulais, voulait, voulu (forme partagée), voudrais (+29 more in data/pilot-300.json)</t>
+          <t>vouloir (forme partagée), veux, veut, voulez (forme partagée), voulais, voulait, voulu (forme partagée), voudrais (+29 autres formes)</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>voir, vu (forme partagée), vois, voit, voyez, voyait, voyons, vue (forme partagée) (+26 more in data/pilot-300.json)</t>
+          <t>voir, vu (forme partagée), vois, voit, voyez, voyait, voyons, vue (forme partagée) (+26 autres formes)</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>savoir (forme partagée), sais (forme partagée), sait, savez, savais, savait, su (forme partagée), savent (+32 more in data/pilot-300.json)</t>
+          <t>savoir (forme partagée), sais (forme partagée), sait, savez, savais, savait, su (forme partagée), savent (+32 autres formes)</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>devoir (forme partagée), dois, doit (forme partagée), dû (forme partagée), devait, devrais, devrait, devez (+30 more in data/pilot-300.json)</t>
+          <t>devoir (forme partagée), dois, doit (forme partagée), dû (forme partagée), devait, devrais, devrait, devez (+30 autres formes)</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>venir, viens, vient, venu (forme partagée), venez, venait, venue (forme partagée), viennent (+27 more in data/pilot-300.json)</t>
+          <t>venir, viens, vient, venu (forme partagée), venez, venait, venue (forme partagée), viennent (+27 autres formes)</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>prendre, pris (forme partagée), prends, prend, prenez, prit, prenait, prise (forme partagée) (+28 more in data/pilot-300.json)</t>
+          <t>prendre, pris (forme partagée), prends, prend, prenez, prit, prenait, prise (forme partagée) (+28 autres formes)</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>parler (forme partagée), parle, parlé (forme partagée), parlait, parles, parlez, parlons, parlent (+27 more in data/pilot-300.json)</t>
+          <t>parler (forme partagée), parle, parlé (forme partagée), parlait, parles, parlez, parlons, parlent (+27 autres formes)</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>suivre, suis (forme partagée), suivi (forme partagée), suivez, suit, suivait, suivit, suivant (forme partagée) (+26 more in data/pilot-300.json)</t>
+          <t>suivre, suis (forme partagée), suivi (forme partagée), suivez, suit, suivait, suivit, suivant (forme partagée) (+26 autres formes)</t>
         </is>
       </c>
       <c r="F78" s="5" t="inlineStr">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>passer (forme partagée), passe (forme partagée), passé (forme partagée), passait, passa, passant (forme partagée), passent, passez (+26 more in data/pilot-300.json)</t>
+          <t>passer (forme partagée), passe (forme partagée), passé (forme partagée), passait, passa, passant (forme partagée), passent, passez (+26 autres formes)</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>croire, crois, croyais, croyez, cru (forme partagée), croit, croyait, croient (+28 more in data/pilot-300.json)</t>
+          <t>croire, crois, croyais, croyez, cru (forme partagée), croit, croyait, croient (+28 autres formes)</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>aimer, aime, aimerais, aimes, aimait, aimé (forme partagée), aimais, aimez (+28 more in data/pilot-300.json)</t>
+          <t>aimer, aime, aimerais, aimes, aimait, aimé (forme partagée), aimais, aimez (+28 autres formes)</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="E100" s="5" t="inlineStr">
         <is>
-          <t>penser, pense, pensais, pensé, penses, pensez, pensait, pensa (+24 more in data/pilot-300.json)</t>
+          <t>penser, pense, pensais, pensé, penses, pensez, pensait, pensa (+24 autres formes)</t>
         </is>
       </c>
       <c r="F100" s="5" t="inlineStr">
@@ -3546,7 +3546,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>trouver, trouvé (forme partagée), trouve, trouvait, trouves, trouvez, trouva, trouvée (forme partagée) (+27 more in data/pilot-300.json)</t>
+          <t>trouver, trouvé (forme partagée), trouve, trouvait, trouves, trouvez, trouva, trouvée (forme partagée) (+27 autres formes)</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="E109" s="6" t="inlineStr">
         <is>
-          <t>regarder, regarde, regardez, regardait, regarda, regardé, regardant (forme partagée), regardais (+24 more in data/pilot-300.json)</t>
+          <t>regarder, regarde, regardez, regardait, regarda, regardé, regardant (forme partagée), regardais (+24 autres formes)</t>
         </is>
       </c>
       <c r="F109" s="6" t="inlineStr">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>laisser, laisse (forme partagée), laissez, laissé (forme partagée), laissait, laissa, laissant, laisses (forme partagée) (+25 more in data/pilot-300.json)</t>
+          <t>laisser, laisse (forme partagée), laissez, laissé (forme partagée), laissait, laissa, laissant, laisses (forme partagée) (+25 autres formes)</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>donner (forme partagée), donne (forme partagée), donné (forme partagée), donnait, donnez, donna, donnent, donnes (forme partagée) (+26 more in data/pilot-300.json)</t>
+          <t>donner (forme partagée), donne (forme partagée), donné (forme partagée), donnait, donnez, donna, donnent, donnes (forme partagée) (+26 autres formes)</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="E114" s="5" t="inlineStr">
         <is>
-          <t>mettre, mis (forme partagée), mit, mets (forme partagée), met, mettez, mettait, mise (forme partagée) (+26 more in data/pilot-300.json)</t>
+          <t>mettre, mis (forme partagée), mit, mets (forme partagée), met, mettez, mettait, mise (forme partagée) (+26 autres formes)</t>
         </is>
       </c>
       <c r="F114" s="5" t="inlineStr">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="E115" s="6" t="inlineStr">
         <is>
-          <t>attendre, attends, attendez, attend, attendait, attendant (forme partagée), attendais, attendu (forme partagée) (+28 more in data/pilot-300.json)</t>
+          <t>attendre, attends, attendez, attend, attendait, attendant (forme partagée), attendais, attendu (forme partagée) (+28 autres formes)</t>
         </is>
       </c>
       <c r="F115" s="6" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="E119" s="6" t="inlineStr">
         <is>
-          <t>arriver, arrive, arrivé (forme partagée), arrivait, arrivent, arrivera, arrivée (forme partagée), arrivés (forme partagée) (+27 more in data/pilot-300.json)</t>
+          <t>arriver, arrive, arrivé (forme partagée), arrivait, arrivent, arrivera, arrivée (forme partagée), arrivés (forme partagée) (+27 autres formes)</t>
         </is>
       </c>
       <c r="F119" s="6" t="inlineStr">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="E121" s="6" t="inlineStr">
         <is>
-          <t>demander, demande (forme partagée), demandé, demanda, demandait, demandais, demandez, demandes (forme partagée) (+23 more in data/pilot-300.json)</t>
+          <t>demander, demande (forme partagée), demandé, demanda, demandait, demandais, demandez, demandes (forme partagée) (+23 autres formes)</t>
         </is>
       </c>
       <c r="F121" s="6" t="inlineStr">
@@ -4102,7 +4102,7 @@
       </c>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>rester, reste (forme partagée), restait, restez, resté, resta, restes (forme partagée), restée (+26 more in data/pilot-300.json)</t>
+          <t>rester, reste (forme partagée), restait, restez, resté, resta, restes (forme partagée), restée (+26 autres formes)</t>
         </is>
       </c>
       <c r="F125" s="6" t="inlineStr">
@@ -4342,7 +4342,7 @@
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>appeler, appelle, appelé (forme partagée), appelait, appelez, appelles, appellent, appelée (+23 more in data/pilot-300.json)</t>
+          <t>appeler, appelle, appelé (forme partagée), appelait, appelez, appelles, appellent, appelée (+23 autres formes)</t>
         </is>
       </c>
       <c r="F133" s="6" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="E136" s="5" t="inlineStr">
         <is>
-          <t>partir, parti (forme partagée), pars (forme partagée), partie (forme partagée), part (forme partagée), partez, partis (forme partagée), partons (+27 more in data/pilot-300.json)</t>
+          <t>partir, parti (forme partagée), pars (forme partagée), partie (forme partagée), part (forme partagée), partez, partis (forme partagée), partons (+27 autres formes)</t>
         </is>
       </c>
       <c r="F136" s="5" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="E137" s="6" t="inlineStr">
         <is>
-          <t>connaître, connais (forme partagée), connaît, connu (forme partagée), connaissez, connaissait, connaissais, connaissent (+28 more in data/pilot-300.json)</t>
+          <t>connaître, connais (forme partagée), connaît, connu (forme partagée), connaissez, connaissait, connaissais, connaissent (+28 autres formes)</t>
         </is>
       </c>
       <c r="F137" s="6" t="inlineStr">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>sortir (forme partagée), sors, sorti, sort (forme partagée), sortez, sortit, sortait, sortie (forme partagée) (+25 more in data/pilot-300.json)</t>
+          <t>sortir (forme partagée), sors, sorti, sort (forme partagée), sortez, sortit, sortait, sortie (forme partagée) (+25 autres formes)</t>
         </is>
       </c>
       <c r="F144" s="5" t="inlineStr">
@@ -4690,7 +4690,7 @@
       </c>
       <c r="E145" s="6" t="inlineStr">
         <is>
-          <t>comprendre, comprends, compris (forme partagée), comprenez, comprend, comprenait, comprit, comprenais (+25 more in data/pilot-300.json)</t>
+          <t>comprendre, comprends, compris (forme partagée), comprenez, comprend, comprenait, comprit, comprenais (+25 autres formes)</t>
         </is>
       </c>
       <c r="F145" s="6" t="inlineStr">
@@ -4778,7 +4778,7 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>arrêter, arrête, arrêtez, arrêté (forme partagée), arrêta, arrêtait, arrêtée (forme partagée), arrêtes (+25 more in data/pilot-300.json)</t>
+          <t>arrêter, arrête, arrêtez, arrêté (forme partagée), arrêta, arrêtait, arrêtée (forme partagée), arrêtes (+25 autres formes)</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>entendre, entendu (forme partagée), entends, entend, entendait, entendit, entendez, entendais (+28 more in data/pilot-300.json)</t>
+          <t>entendre, entendu (forme partagée), entends, entend, entendait, entendit, entendez, entendais (+28 autres formes)</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
@@ -5138,7 +5138,7 @@
       </c>
       <c r="E160" s="5" t="inlineStr">
         <is>
-          <t>mourir, mort (forme partagée), morte (forme partagée), morts (forme partagée), meurt, meurs, meurent, meure (+27 more in data/pilot-300.json)</t>
+          <t>mourir, mort (forme partagée), morte (forme partagée), morts (forme partagée), meurt, meurs, meurent, meure (+27 autres formes)</t>
         </is>
       </c>
       <c r="F160" s="5" t="inlineStr">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="E165" s="6" t="inlineStr">
         <is>
-          <t>sentir, sens (forme partagée), sentait, sent, sentais, senti (forme partagée), sentit, sentez (+26 more in data/pilot-300.json)</t>
+          <t>sentir, sens (forme partagée), sentait, sent, sentais, senti (forme partagée), sentit, sentez (+26 autres formes)</t>
         </is>
       </c>
       <c r="F165" s="6" t="inlineStr">
@@ -5314,7 +5314,7 @@
       </c>
       <c r="E166" s="5" t="inlineStr">
         <is>
-          <t>tenir, tenait, tient, tiens (forme partagée), tenez, tenu (forme partagée), tenant (forme partagée), tenaient (+26 more in data/pilot-300.json)</t>
+          <t>tenir, tenait, tient, tiens (forme partagée), tenez, tenu (forme partagée), tenant (forme partagée), tenaient (+26 autres formes)</t>
         </is>
       </c>
       <c r="F166" s="5" t="inlineStr">
@@ -5662,7 +5662,7 @@
       </c>
       <c r="E178" s="5" t="inlineStr">
         <is>
-          <t>chercher, cherche, cherchait, cherché, cherchez, cherches, cherchais, cherchant (+25 more in data/pilot-300.json)</t>
+          <t>chercher, cherche, cherchait, cherché, cherchez, cherches, cherchais, cherchant (+25 autres formes)</t>
         </is>
       </c>
       <c r="F178" s="5" t="inlineStr">
@@ -5810,7 +5810,7 @@
       </c>
       <c r="E183" s="6" t="inlineStr">
         <is>
-          <t>revenir, reviens, revient (forme partagée), revenu (forme partagée), revint, revenait, reviendra, revenue (forme partagée) (+26 more in data/pilot-300.json)</t>
+          <t>revenir, reviens, revient (forme partagée), revenu (forme partagée), revint, revenait, reviendra, revenue (forme partagée) (+26 autres formes)</t>
         </is>
       </c>
       <c r="F183" s="6" t="inlineStr">
@@ -5926,7 +5926,7 @@
       </c>
       <c r="E187" s="6" t="inlineStr">
         <is>
-          <t>tuer, tué (forme partagée), tue (forme partagée), tuée (forme partagée), tuez, tués (forme partagée), tuerai, tuera (+23 more in data/pilot-300.json)</t>
+          <t>tuer, tué (forme partagée), tue (forme partagée), tuée (forme partagée), tuez, tués (forme partagée), tuerai, tuera (+23 autres formes)</t>
         </is>
       </c>
       <c r="F187" s="6" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="E206" s="5" t="inlineStr">
         <is>
-          <t>rendre, rend, rends, rendu (forme partagée), rendait, rendez, rendit, rendent (+27 more in data/pilot-300.json)</t>
+          <t>rendre, rend, rends, rendu (forme partagée), rendait, rendez, rendit, rendent (+27 autres formes)</t>
         </is>
       </c>
       <c r="F206" s="5" t="inlineStr">
@@ -6502,7 +6502,7 @@
       </c>
       <c r="E207" s="6" t="inlineStr">
         <is>
-          <t>finir, fini (forme partagée), finit, finie (forme partagée), finis (forme partagée), finissait, finira, finissent (+23 more in data/pilot-300.json)</t>
+          <t>finir, fini (forme partagée), finit, finie (forme partagée), finis (forme partagée), finissait, finira, finissent (+23 autres formes)</t>
         </is>
       </c>
       <c r="F207" s="6" t="inlineStr">
@@ -6530,7 +6530,7 @@
       </c>
       <c r="E208" s="5" t="inlineStr">
         <is>
-          <t>devenir (forme partagée), devenu, devient, devenue, devenait, deviens, devenus, devint (+29 more in data/pilot-300.json)</t>
+          <t>devenir (forme partagée), devenu, devient, devenue, devenait, deviens, devenus, devint (+29 autres formes)</t>
         </is>
       </c>
       <c r="F208" s="5" t="inlineStr">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="E209" s="6" t="inlineStr">
         <is>
-          <t>vivre (forme partagée), vit (forme partagée), vécu (forme partagée), vivait, vivent, vis (forme partagée), vivaient, vivons (+26 more in data/pilot-300.json)</t>
+          <t>vivre (forme partagée), vit (forme partagée), vécu (forme partagée), vivait, vivent, vis (forme partagée), vivaient, vivons (+26 autres formes)</t>
         </is>
       </c>
       <c r="F209" s="6" t="inlineStr">
@@ -6586,7 +6586,7 @@
       </c>
       <c r="E210" s="5" t="inlineStr">
         <is>
-          <t>essayer, essaie, essayé, essaye, essayez, essayait, essayais, essayant (+37 more in data/pilot-300.json)</t>
+          <t>essayer, essaie, essayé, essaye, essayez, essayait, essayais, essayant (+37 autres formes)</t>
         </is>
       </c>
       <c r="F210" s="5" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="E215" s="6" t="inlineStr">
         <is>
-          <t>perdre, perdu (forme partagée), perd, perds, perdue (forme partagée), perdait, perdus (forme partagée), perdez (+27 more in data/pilot-300.json)</t>
+          <t>perdre, perdu (forme partagée), perd, perds, perdue (forme partagée), perdait, perdus (forme partagée), perdez (+27 autres formes)</t>
         </is>
       </c>
       <c r="F215" s="6" t="inlineStr">
@@ -6822,7 +6822,7 @@
       </c>
       <c r="E218" s="5" t="inlineStr">
         <is>
-          <t>jouer, joue (forme partagée), joué (forme partagée), jouait, joues (forme partagée), jouent, jouez, jouant (+24 more in data/pilot-300.json)</t>
+          <t>jouer, joue (forme partagée), joué (forme partagée), jouait, joues (forme partagée), jouent, jouez, jouant (+24 autres formes)</t>
         </is>
       </c>
       <c r="F218" s="5" t="inlineStr">
@@ -6850,7 +6850,7 @@
       </c>
       <c r="E219" s="6" t="inlineStr">
         <is>
-          <t>ouvrir, ouvre, ouvert (forme partagée), ouvrit, ouvrez, ouverte (forme partagée), ouvrait, ouvrant (forme partagée) (+25 more in data/pilot-300.json)</t>
+          <t>ouvrir, ouvre, ouvert (forme partagée), ouvrit, ouvrez, ouverte (forme partagée), ouvrait, ouvrant (forme partagée) (+25 autres formes)</t>
         </is>
       </c>
       <c r="F219" s="6" t="inlineStr">
@@ -7170,7 +7170,7 @@
       </c>
       <c r="E230" s="5" t="inlineStr">
         <is>
-          <t>commencer, commence, commencé, commençait, commença, commencent, commençaient, commençais (+25 more in data/pilot-300.json)</t>
+          <t>commencer, commence, commencé, commençait, commença, commencent, commençaient, commençais (+25 autres formes)</t>
         </is>
       </c>
       <c r="F230" s="5" t="inlineStr">
@@ -7230,7 +7230,7 @@
       </c>
       <c r="E232" s="5" t="inlineStr">
         <is>
-          <t>tomber, tombe (forme partagée), tombé (forme partagée), tombée (forme partagée), tombait, tomba, tombent, tombés (forme partagée) (+24 more in data/pilot-300.json)</t>
+          <t>tomber, tombe (forme partagée), tombé (forme partagée), tombée (forme partagée), tombait, tomba, tombent, tombés (forme partagée) (+24 autres formes)</t>
         </is>
       </c>
       <c r="F232" s="5" t="inlineStr">
@@ -7258,7 +7258,7 @@
       </c>
       <c r="E233" s="6" t="inlineStr">
         <is>
-          <t>entrer, entre (forme partagée), entrez, entré, entra, entrait, entrée (forme partagée), entrés (+25 more in data/pilot-300.json)</t>
+          <t>entrer, entre (forme partagée), entrez, entré, entra, entrait, entrée (forme partagée), entrés (+25 autres formes)</t>
         </is>
       </c>
       <c r="F233" s="6" t="inlineStr">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="E234" s="5" t="inlineStr">
         <is>
-          <t>aider, aide (forme partagée), aidez, aidé, aidera, aides (forme partagée), aidée, aidait (+24 more in data/pilot-300.json)</t>
+          <t>aider, aide (forme partagée), aidez, aidé, aidera, aides (forme partagée), aidée, aidait (+24 autres formes)</t>
         </is>
       </c>
       <c r="F234" s="5" t="inlineStr">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="E243" s="6" t="inlineStr">
         <is>
-          <t>rentrer, rentre, rentré (forme partagée), rentrée (forme partagée), rentrez, rentrant (forme partagée), rentres, rentrons (+24 more in data/pilot-300.json)</t>
+          <t>rentrer, rentre, rentré (forme partagée), rentrée (forme partagée), rentrez, rentrant (forme partagée), rentres, rentrons (+24 autres formes)</t>
         </is>
       </c>
       <c r="F243" s="6" t="inlineStr">
@@ -7630,7 +7630,7 @@
       </c>
       <c r="E246" s="5" t="inlineStr">
         <is>
-          <t>sembler, semblait, semble, semblaient, semblent, sembla, semblé, semblant (forme partagée) (+12 more in data/pilot-300.json)</t>
+          <t>sembler, semblait, semble, semblaient, semblent, sembla, semblé, semblant (forme partagée) (+12 autres formes)</t>
         </is>
       </c>
       <c r="F246" s="5" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="E249" s="6" t="inlineStr">
         <is>
-          <t>tirer, tire (forme partagée), tiré (forme partagée), tirez, tira, tirait, tirant (forme partagée), tirent (+25 more in data/pilot-300.json)</t>
+          <t>tirer, tire (forme partagée), tiré (forme partagée), tirez, tira, tirait, tirant (forme partagée), tirent (+25 autres formes)</t>
         </is>
       </c>
       <c r="F249" s="6" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="E251" s="6" t="inlineStr">
         <is>
-          <t>porter (forme partagée), porte (forme partagée), portait, porté, portant (forme partagée), portaient, portent, portes (forme partagée) (+24 more in data/pilot-300.json)</t>
+          <t>porter (forme partagée), porte (forme partagée), portait, porté, portant (forme partagée), portaient, portent, portes (forme partagée) (+24 autres formes)</t>
         </is>
       </c>
       <c r="F251" s="6" t="inlineStr">
@@ -7802,7 +7802,7 @@
       </c>
       <c r="E252" s="5" t="inlineStr">
         <is>
-          <t>écouter, écoute (forme partagée), écoutez, écoutait, écouté, écoutes (forme partagée), écoutant (forme partagée), écoutais (+23 more in data/pilot-300.json)</t>
+          <t>écouter, écoute (forme partagée), écoutez, écoutait, écouté, écoutes (forme partagée), écoutant (forme partagée), écoutais (+23 autres formes)</t>
         </is>
       </c>
       <c r="F252" s="5" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="E254" s="5" t="inlineStr">
         <is>
-          <t>oublier, oublié (forme partagée), oublie (forme partagée), oubliez, oublierai, oublies (forme partagée), oubliais, oubliée (forme partagée) (+25 more in data/pilot-300.json)</t>
+          <t>oublier, oublié (forme partagée), oublie (forme partagée), oubliez, oublierai, oublies (forme partagée), oubliais, oubliée (forme partagée) (+25 autres formes)</t>
         </is>
       </c>
       <c r="F254" s="5" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="E261" s="6" t="inlineStr">
         <is>
-          <t>manger (forme partagée), mange, mangé, mangeait, manges, mangent, mangez, mangeant (+26 more in data/pilot-300.json)</t>
+          <t>manger (forme partagée), mange, mangé, mangeait, manges, mangent, mangez, mangeant (+26 autres formes)</t>
         </is>
       </c>
       <c r="F261" s="6" t="inlineStr">
@@ -8130,7 +8130,7 @@
       </c>
       <c r="E263" s="6" t="inlineStr">
         <is>
-          <t>plaire, plaît, plaisait, plais, plairait, plaira, plaisent, plaise (+20 more in data/pilot-300.json)</t>
+          <t>plaire, plaît, plaisait, plais, plairait, plaira, plaisent, plaise (+20 autres formes)</t>
         </is>
       </c>
       <c r="F263" s="6" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>répondre, répondit, répondu, réponds, répond, répondait, répondez, répondis (+23 more in data/pilot-300.json)</t>
+          <t>répondre, répondit, répondu, réponds, répond, répondait, répondez, répondis (+23 autres formes)</t>
         </is>
       </c>
       <c r="F271" s="6" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="E273" s="6" t="inlineStr">
         <is>
-          <t>asseoir, assis (forme partagée), assieds, asseyez, assise (forme partagée), assit, assied, asseyait (+35 more in data/pilot-300.json)</t>
+          <t>asseoir, assis (forme partagée), assieds, asseyez, assise (forme partagée), assit, assied, asseyait (+35 autres formes)</t>
         </is>
       </c>
       <c r="F273" s="6" t="inlineStr">
@@ -8498,7 +8498,7 @@
       </c>
       <c r="E275" s="6" t="inlineStr">
         <is>
-          <t>retrouver, retrouve, retrouvé, retrouvait, retrouva, retrouvée, retrouvés, retrouvera (+25 more in data/pilot-300.json)</t>
+          <t>retrouver, retrouve, retrouvé, retrouvait, retrouva, retrouvée, retrouvés, retrouvera (+25 autres formes)</t>
         </is>
       </c>
       <c r="F275" s="6" t="inlineStr">
@@ -8854,7 +8854,7 @@
       </c>
       <c r="E287" s="6" t="inlineStr">
         <is>
-          <t>marcher, marche (forme partagée), marché (forme partagée), marchait, marchant (forme partagée), marchent, marcha, marchera (+23 more in data/pilot-300.json)</t>
+          <t>marcher, marche (forme partagée), marché (forme partagée), marchait, marchant (forme partagée), marchent, marcha, marchera (+23 autres formes)</t>
         </is>
       </c>
       <c r="F287" s="6" t="inlineStr">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="E289" s="6" t="inlineStr">
         <is>
-          <t>travailler, travaille, travaillé (forme partagée), travaillait, travaillent, travaillez, travailles, travaillais (+25 more in data/pilot-300.json)</t>
+          <t>travailler, travaille, travaillé (forme partagée), travaillait, travaillent, travaillez, travailles, travaillais (+25 autres formes)</t>
         </is>
       </c>
       <c r="F289" s="6" t="inlineStr">
@@ -8942,7 +8942,7 @@
       </c>
       <c r="E290" s="5" t="inlineStr">
         <is>
-          <t>monter, monte, montait, monté (forme partagée), monta, montaient, montée (forme partagée), montent (+23 more in data/pilot-300.json)</t>
+          <t>monter, monte, montait, monté (forme partagée), monta, montaient, montée (forme partagée), montent (+23 autres formes)</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
@@ -9090,7 +9090,7 @@
       </c>
       <c r="E295" s="6" t="inlineStr">
         <is>
-          <t>changer, changé (forme partagée), change (forme partagée), changera, changeait, changent, changea, changez (+24 more in data/pilot-300.json)</t>
+          <t>changer, changé (forme partagée), change (forme partagée), changera, changeait, changent, changea, changez (+24 autres formes)</t>
         </is>
       </c>
       <c r="F295" s="6" t="inlineStr">
@@ -9150,7 +9150,7 @@
       </c>
       <c r="E297" s="6" t="inlineStr">
         <is>
-          <t>dormir, dort, dors, dormi, dormait, dormais, dorment, dormez (+23 more in data/pilot-300.json)</t>
+          <t>dormir, dort, dors, dormi, dormait, dormais, dorment, dormez (+23 autres formes)</t>
         </is>
       </c>
       <c r="F297" s="6" t="inlineStr">
@@ -9210,7 +9210,7 @@
       </c>
       <c r="E299" s="6" t="inlineStr">
         <is>
-          <t>écrire, écrit (forme partagée), écris, écrivait, écrivais, écrivez, écrite (forme partagée), écrivit (+25 more in data/pilot-300.json)</t>
+          <t>écrire, écrit (forme partagée), écris, écrivait, écrivais, écrivez, écrite (forme partagée), écrivit (+25 autres formes)</t>
         </is>
       </c>
       <c r="F299" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Record French teacher review artifacts and diagnostics
</commit_message>
<xml_diff>
--- a/data/review-sheet.xlsx
+++ b/data/review-sheet.xlsx
@@ -10,10 +10,13 @@
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Mots" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="À revérifier" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Mots'!$A$1:$H$301</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Changes'!$A$1:$E$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'À revérifier'!$A$1:$G$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -85,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -106,6 +109,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2840,7 +2846,7 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>la chose</t>
+          <t>chose</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -3300,7 +3306,7 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>le jour</t>
+          <t>jour</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
@@ -3448,7 +3454,7 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>le temps</t>
+          <t>temps</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
@@ -3788,7 +3794,7 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>la femme</t>
+          <t>femme</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -3820,7 +3826,7 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>la fois</t>
+          <t>fois</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
@@ -3908,7 +3914,7 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>le peu</t>
+          <t>peu</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
@@ -4000,7 +4006,7 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>la vie</t>
+          <t>vie</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -4092,7 +4098,7 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>la main</t>
+          <t>main</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
@@ -4300,7 +4306,7 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>le père</t>
+          <t>père</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
@@ -4416,7 +4422,7 @@
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>le monde</t>
+          <t>monde</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
@@ -4736,7 +4742,7 @@
       </c>
       <c r="B147" s="6" t="inlineStr">
         <is>
-          <t>la mère</t>
+          <t>mère</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
@@ -4824,7 +4830,7 @@
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
-          <t>la fille</t>
+          <t>fille</t>
         </is>
       </c>
       <c r="C150" s="5" t="inlineStr">
@@ -4884,7 +4890,7 @@
       </c>
       <c r="B152" s="5" t="inlineStr">
         <is>
-          <t>la tête</t>
+          <t>tête</t>
         </is>
       </c>
       <c r="C152" s="5" t="inlineStr">
@@ -5004,7 +5010,7 @@
       </c>
       <c r="B156" s="5" t="inlineStr">
         <is>
-          <t>la nuit</t>
+          <t>nuit</t>
         </is>
       </c>
       <c r="C156" s="5" t="inlineStr">
@@ -5036,7 +5042,7 @@
       </c>
       <c r="B157" s="6" t="inlineStr">
         <is>
-          <t>le coup</t>
+          <t>coup</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
@@ -5152,7 +5158,7 @@
       </c>
       <c r="B161" s="6" t="inlineStr">
         <is>
-          <t>le dieu</t>
+          <t>dieu</t>
         </is>
       </c>
       <c r="C161" s="6" t="inlineStr">
@@ -5500,7 +5506,7 @@
       </c>
       <c r="B173" s="6" t="inlineStr">
         <is>
-          <t>la maison</t>
+          <t>maison</t>
         </is>
       </c>
       <c r="C173" s="6" t="inlineStr">
@@ -5592,7 +5598,7 @@
       </c>
       <c r="B176" s="5" t="inlineStr">
         <is>
-          <t>le soir</t>
+          <t>soir</t>
         </is>
       </c>
       <c r="C176" s="5" t="inlineStr">
@@ -5680,7 +5686,7 @@
       </c>
       <c r="B179" s="6" t="inlineStr">
         <is>
-          <t>le moment</t>
+          <t>moment</t>
         </is>
       </c>
       <c r="C179" s="6" t="inlineStr">
@@ -5996,7 +6002,7 @@
       </c>
       <c r="B190" s="5" t="inlineStr">
         <is>
-          <t>le monsieur</t>
+          <t>monsieur</t>
         </is>
       </c>
       <c r="C190" s="5" t="inlineStr">
@@ -6200,7 +6206,7 @@
       </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
-          <t>le besoin</t>
+          <t>besoin</t>
         </is>
       </c>
       <c r="C197" s="6" t="inlineStr">
@@ -6288,7 +6294,7 @@
       </c>
       <c r="B200" s="5" t="inlineStr">
         <is>
-          <t>le les gens</t>
+          <t>les gens</t>
         </is>
       </c>
       <c r="C200" s="5" t="inlineStr">
@@ -6516,7 +6522,7 @@
       </c>
       <c r="B208" s="5" t="inlineStr">
         <is>
-          <t>le nom</t>
+          <t>nom</t>
         </is>
       </c>
       <c r="C208" s="5" t="inlineStr">
@@ -6576,7 +6582,7 @@
       </c>
       <c r="B210" s="5" t="inlineStr">
         <is>
-          <t>la porte</t>
+          <t>porte</t>
         </is>
       </c>
       <c r="C210" s="5" t="inlineStr">
@@ -6692,7 +6698,7 @@
       </c>
       <c r="B214" s="5" t="inlineStr">
         <is>
-          <t>la mort</t>
+          <t>mort</t>
         </is>
       </c>
       <c r="C214" s="5" t="inlineStr">
@@ -6980,7 +6986,7 @@
       </c>
       <c r="B224" s="5" t="inlineStr">
         <is>
-          <t>la peur</t>
+          <t>peur</t>
         </is>
       </c>
       <c r="C224" s="5" t="inlineStr">
@@ -7100,7 +7106,7 @@
       </c>
       <c r="B228" s="5" t="inlineStr">
         <is>
-          <t>le côté</t>
+          <t>côté</t>
         </is>
       </c>
       <c r="C228" s="5" t="inlineStr">
@@ -7304,7 +7310,7 @@
       </c>
       <c r="B235" s="6" t="inlineStr">
         <is>
-          <t>le mot</t>
+          <t>mot</t>
         </is>
       </c>
       <c r="C235" s="6" t="inlineStr">
@@ -7704,7 +7710,7 @@
       </c>
       <c r="B249" s="6" t="inlineStr">
         <is>
-          <t>la raison</t>
+          <t>raison</t>
         </is>
       </c>
       <c r="C249" s="6" t="inlineStr">
@@ -7764,7 +7770,7 @@
       </c>
       <c r="B251" s="6" t="inlineStr">
         <is>
-          <t>la place</t>
+          <t>place</t>
         </is>
       </c>
       <c r="C251" s="6" t="inlineStr">
@@ -7796,7 +7802,7 @@
       </c>
       <c r="B252" s="5" t="inlineStr">
         <is>
-          <t>le fait</t>
+          <t>fait</t>
         </is>
       </c>
       <c r="C252" s="5" t="inlineStr">
@@ -7972,7 +7978,7 @@
       </c>
       <c r="B258" s="5" t="inlineStr">
         <is>
-          <t>la terre</t>
+          <t>terre</t>
         </is>
       </c>
       <c r="C258" s="5" t="inlineStr">
@@ -8032,7 +8038,7 @@
       </c>
       <c r="B260" s="5" t="inlineStr">
         <is>
-          <t>la voix</t>
+          <t>voix</t>
         </is>
       </c>
       <c r="C260" s="5" t="inlineStr">
@@ -8064,7 +8070,7 @@
       </c>
       <c r="B261" s="6" t="inlineStr">
         <is>
-          <t>la question</t>
+          <t>question</t>
         </is>
       </c>
       <c r="C261" s="6" t="inlineStr">
@@ -8124,7 +8130,7 @@
       </c>
       <c r="B263" s="6" t="inlineStr">
         <is>
-          <t>le corps</t>
+          <t>corps</t>
         </is>
       </c>
       <c r="C263" s="6" t="inlineStr">
@@ -8156,7 +8162,7 @@
       </c>
       <c r="B264" s="5" t="inlineStr">
         <is>
-          <t>le fils</t>
+          <t>fils</t>
         </is>
       </c>
       <c r="C264" s="5" t="inlineStr">
@@ -8188,7 +8194,7 @@
       </c>
       <c r="B265" s="6" t="inlineStr">
         <is>
-          <t>la rue</t>
+          <t>rue</t>
         </is>
       </c>
       <c r="C265" s="6" t="inlineStr">
@@ -8340,7 +8346,7 @@
       </c>
       <c r="B270" s="5" t="inlineStr">
         <is>
-          <t>la voiture</t>
+          <t>voiture</t>
         </is>
       </c>
       <c r="C270" s="5" t="inlineStr">
@@ -8516,7 +8522,7 @@
       </c>
       <c r="B276" s="5" t="inlineStr">
         <is>
-          <t>le visage</t>
+          <t>visage</t>
         </is>
       </c>
       <c r="C276" s="5" t="inlineStr">
@@ -8576,7 +8582,7 @@
       </c>
       <c r="B278" s="5" t="inlineStr">
         <is>
-          <t>la chambre</t>
+          <t>chambre</t>
         </is>
       </c>
       <c r="C278" s="5" t="inlineStr">
@@ -8636,7 +8642,7 @@
       </c>
       <c r="B280" s="5" t="inlineStr">
         <is>
-          <t>le pied</t>
+          <t>pied</t>
         </is>
       </c>
       <c r="C280" s="5" t="inlineStr">
@@ -8756,7 +8762,7 @@
       </c>
       <c r="B284" s="5" t="inlineStr">
         <is>
-          <t>la maman</t>
+          <t>maman</t>
         </is>
       </c>
       <c r="C284" s="5" t="inlineStr">
@@ -8900,7 +8906,7 @@
       </c>
       <c r="B289" s="6" t="inlineStr">
         <is>
-          <t>le matin</t>
+          <t>matin</t>
         </is>
       </c>
       <c r="C289" s="6" t="inlineStr">
@@ -8932,7 +8938,7 @@
       </c>
       <c r="B290" s="5" t="inlineStr">
         <is>
-          <t>la famille</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C290" s="5" t="inlineStr">
@@ -8992,7 +8998,7 @@
       </c>
       <c r="B292" s="5" t="inlineStr">
         <is>
-          <t>le travail</t>
+          <t>travail</t>
         </is>
       </c>
       <c r="C292" s="5" t="inlineStr">
@@ -9052,7 +9058,7 @@
       </c>
       <c r="B294" s="5" t="inlineStr">
         <is>
-          <t>la ville</t>
+          <t>ville</t>
         </is>
       </c>
       <c r="C294" s="5" t="inlineStr">
@@ -9172,7 +9178,7 @@
       </c>
       <c r="B298" s="5" t="inlineStr">
         <is>
-          <t>le cœur</t>
+          <t>cœur</t>
         </is>
       </c>
       <c r="C298" s="5" t="inlineStr">
@@ -9204,7 +9210,7 @@
       </c>
       <c r="B299" s="6" t="inlineStr">
         <is>
-          <t>le bras</t>
+          <t>bras</t>
         </is>
       </c>
       <c r="C299" s="6" t="inlineStr">
@@ -9264,18 +9270,22 @@
       </c>
       <c r="B301" s="6" t="inlineStr">
         <is>
-          <t>bon</t>
-        </is>
-      </c>
-      <c r="C301" s="6" t="inlineStr"/>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="C301" s="6" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="D301" s="6" t="inlineStr">
         <is>
-          <t>onomatopée</t>
+          <t>adjectif</t>
         </is>
       </c>
       <c r="E301" s="6" t="inlineStr">
         <is>
-          <t>bon (forme partagée)</t>
+          <t>noir (forme partagée), noire (forme partagée), noirs (forme partagée), noires (forme partagée)</t>
         </is>
       </c>
       <c r="F301" s="6" t="inlineStr">
@@ -10397,4 +10407,1286 @@
   <autoFilter ref="A1:E43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Sujet</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>Demandes de vérification POS hors des 300 mots classés</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Ces demandes sont conservées ici pour ne pas ajouter de lignes au CSV des 300 mots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>le peu</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Confirmé par l'enseignante</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>bonjour</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Note POS : code à confirmer ; entrée hors des 300 mots classés.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Mot</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Formes</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Avis</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Correction</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>je</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr"/>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>pronom personnel</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>je, j'</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>adverbe</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>ne, n'</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>me</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>pronom personnel</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>me, m'</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>pronom démonstratif</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>ce, c'</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>que</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>pronom interrogatif</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>que, qu'</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>que</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>pronom relatif</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>que, qu'</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>tout</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr"/>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>adjectif indéfini</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>tout, tous, toute, toutes</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>tout</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>pronom indéfini</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>tout, tous</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>le</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>pronom personnel</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>le, l'</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>la</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>pronom personnel</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>la, l'</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>où</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr"/>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>adverbe</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>où</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>falloir</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr"/>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>verbe</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>faut, fallait, faudrait, faudra, fallu, falloir, fallut, faille</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>conjonction</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>si, s'</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>quoi</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr"/>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>adjectif</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>dont</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>pronom interrogatif</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>conjonction</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>est-ce que</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>locution interrogative</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>est-ce que, est-ce qu'</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>beau</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>adjectif</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>beau, belle, beaux, belles, bel</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>autre</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr"/>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>pronom indéfini</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>autre, autres</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>leur / leurs</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>adjectif possessif</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>leurs, leur</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>leur</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>pronom possessif</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>leur, leurs</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>quel</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr"/>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>adjectif interrogatif</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>quel, quelles, quels</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr"/>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>pronom indéfini</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>un, une, unes, uns</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>parce que</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>conjonction</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>parce que, parce qu'</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>vieux</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>adjectif</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>vieux, vieille, vieilles, vieil</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>mort</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>mort, morts</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>l'œil</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>yeux, œil</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>l'homme</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>homme, hommes</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>l'heure</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>heure, heures</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>l'an</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>ans, an</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>l'enfant</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>m/f</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>enfants, enfant</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>l'air</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>air, airs</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="7" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>l'ami(e)</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>m/f</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>ami, amis, amie, amies</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>les gens</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>gens</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>l'accord</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>accord, accords</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>l'amour</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>amour, amours</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>l'eau</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>eau, eaux</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="7" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>l'histoire</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>histoire, histoires</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="7" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>l'idée</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>idée, idées</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>l'argent</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>argent</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="7" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>l'année</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>années, année</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="n"/>
+      <c r="G42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>l'affaire</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>affaire, affaires</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="7" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>cœur</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>cœur, cœurs</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="n"/>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Réapprovisionnement — rang Lexique 301</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>bras</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>nom</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>bras</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="n"/>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Réapprovisionnement — rang Lexique 302</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>apprendre</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr"/>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>verbe</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>appris, apprendre, apprend, apprends, apprit, apprendra, apprenait, apprennent, apprendrai, apprenne, apprenant, apprenez</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Réapprovisionnement — rang Lexique 303</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>noir</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>adjectif</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>noir, noire, noirs, noires</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="n"/>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Réapprovisionnement — rang Lexique 305</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G47"/>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisissez OK, Faux ou À corriger." type="list">
+      <formula1>"OK,Faux,À corriger"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>